<commit_message>
v1.6.26 订舱单补 LOGO(DETRANS/ANHAI/CHR) + CHR 箱号连续性误报修复
</commit_message>
<xml_diff>
--- a/templates/tpl_booking_mssnhsj6ni6f.xlsx
+++ b/templates/tpl_booking_mssnhsj6ni6f.xlsx
@@ -188,6 +188,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -727,7 +776,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" ht="14.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" ht="14.25" customHeight="1" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>25</v>
       </c>
@@ -802,9 +851,6 @@
       <c r="F28"/>
       <c r="G28"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25"/>
     <row r="32" ht="21.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>35</v>
@@ -843,5 +889,6 @@
     <mergeCell ref="A32:I32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>